<commit_message>
MLB自動更新: 2026-08-25 (steps: all)
</commit_message>
<xml_diff>
--- a/data/MLB/2026年/公式戦/raw/2026-08-25/highlights_20260825.xlsx
+++ b/data/MLB/2026年/公式戦/raw/2026-08-25/highlights_20260825.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,216 +450,6 @@
       <c r="G1" t="inlineStr">
         <is>
           <t>detail</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>カル・ローリー</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>raleigh, cal</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>マリナーズ</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>打者</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>フィリーズ戦で3本塁打を放ち、チームの大量得点に大きく貢献した。</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>アンソニー・シーグラー</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>seigler, anthony</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>レッドソックス</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>打者</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>9回表にマイアミ・マーリンズ相手に逆転のタイムリー三塁打を放ち、劇的な勝利を呼び込んだ。</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>3</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>ニック・ゴンザレス</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>gonzales, nick</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>パイレーツ</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>打者</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>12回表にパドレス相手に勝ち越しのタイムリーヒットを放ち、延長戦の激闘に終止符を打った。</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>クマール・ロッカー</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>rocker, kumar</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>レンジャーズ</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>投手</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>ホワイトソックス相手に5.2回を投げ2失点8奪三振の力投を見せ、試合を支配した。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>5</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>ケビン・ゴーズマン</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>gausman, kevin</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>カブス</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>投手</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>ダイヤモンドバックス相手に6.2回を無失点に抑える好投で、チームを勝利に導いた。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>6</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>ブラクストン・アッシュクラフト</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>ashcraft, braxton</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>パイレーツ</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>投手</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>パドレス相手に6回を無失点に抑える好投で、投手戦の口火を切った。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
MLB自動更新: 2026-08-25:2026-08-26 (steps: highlights)
</commit_message>
<xml_diff>
--- a/data/MLB/2026年/公式戦/raw/2026-08-25/highlights_20260825.xlsx
+++ b/data/MLB/2026年/公式戦/raw/2026-08-25/highlights_20260825.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,6 +450,216 @@
       <c r="G1" t="inlineStr">
         <is>
           <t>detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>カル・ラレー</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>raleigh, cal</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>マリナーズ</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>打者</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>フィリーズ戦でザック・ウィーラーから3本のホームランを放ち、チームの大量得点に大きく貢献した。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>アンソニー・シーグラー</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>seigler, anthony</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>レッドソックス</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>打者</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>9回表にマーリンズのタイラー・ザバーから逆転のタイムリー三塁打を放ち、劇的な勝利を呼び込んだ。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ニック・ゴンザレス</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>gonzales, nick</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>パイレーツ</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>打者</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>12回表にパドレスのブラッドリー・ロドリゲスから勝ち越しのタイムリーヒットを放ち、延長戦を制した。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ケビン・ガウスマン</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>gausman, kevin</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>カブス</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>投手</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>ダイヤモンドバックス相手に6.2回を無失点に抑え、6奪三振の快投で試合を支配した。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ブラクストン・アッシュクラフト</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ashcraft, braxton</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>パイレーツ</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>投手</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>パドレス相手に6回を無失点に抑える好投を見せ、チームの勝利に貢献した。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>サンディ・アルカンタラ</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>alcantara, sandy</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>マーリンズ</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>投手</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>レッドソックス相手に7回1失点6奪三振の安定した投球で試合を作り、チームを牽引した。</t>
         </is>
       </c>
     </row>

</xml_diff>